<commit_message>
excel: ajustar ancho de columnas
</commit_message>
<xml_diff>
--- a/SEMANA09/Semana09_BoletaPago/Excel/Boleta_de_pago_Lab09.xlsx
+++ b/SEMANA09/Semana09_BoletaPago/Excel/Boleta_de_pago_Lab09.xlsx
@@ -597,7 +597,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -1005,7 +1005,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1603,31 +1603,31 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>